<commit_message>
fix(official): update 汇玺III 8座45D and 7座50/51F 5 units discount from 25% to 20% in Excel workbooks and regenerate data
</commit_message>
<xml_diff>
--- a/九龙-西南九龙-汇玺III/汇玺III_销控明细表.xlsx
+++ b/九龙-西南九龙-汇玺III/汇玺III_销控明细表.xlsx
@@ -25603,14 +25603,14 @@
       </c>
       <c r="J403" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="K403" s="5" t="n">
-        <v>7997250</v>
+        <v>8530400</v>
       </c>
       <c r="L403" s="5" t="n">
-        <v>22849</v>
+        <v>24373</v>
       </c>
       <c r="M403" s="3" t="inlineStr">
         <is>
@@ -26099,14 +26099,14 @@
       </c>
       <c r="J411" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="K411" s="5" t="n">
-        <v>8309250</v>
+        <v>8863200</v>
       </c>
       <c r="L411" s="5" t="n">
-        <v>21866</v>
+        <v>23324</v>
       </c>
       <c r="M411" s="3" t="inlineStr">
         <is>
@@ -26161,14 +26161,14 @@
       </c>
       <c r="J412" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="K412" s="5" t="n">
-        <v>8016750</v>
+        <v>8551200</v>
       </c>
       <c r="L412" s="5" t="n">
-        <v>22646</v>
+        <v>24156</v>
       </c>
       <c r="M412" s="3" t="inlineStr">
         <is>
@@ -26223,14 +26223,14 @@
       </c>
       <c r="J413" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="K413" s="5" t="n">
-        <v>7963500</v>
+        <v>8494400</v>
       </c>
       <c r="L413" s="5" t="n">
-        <v>22753</v>
+        <v>24270</v>
       </c>
       <c r="M413" s="3" t="inlineStr">
         <is>
@@ -55867,14 +55867,14 @@
       </c>
       <c r="J891" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="K891" s="5" t="n">
-        <v>6960000</v>
+        <v>7424000</v>
       </c>
       <c r="L891" s="5" t="n">
-        <v>25309</v>
+        <v>26996</v>
       </c>
       <c r="M891" s="3" t="inlineStr">
         <is>
@@ -77356,8 +77356,8 @@
       <c r="H5" s="23" t="inlineStr">
         <is>
           <t>G | 350呎 (1房)
-$1066万
-$30,466/呎
+$853.04万
+$24,373/呎
 (暂停销售)</t>
         </is>
       </c>
@@ -77459,24 +77459,24 @@
       <c r="I6" s="23" t="inlineStr">
         <is>
           <t>H | 350呎 (1房)
-$1062万
-$30,337/呎
+$849.44万
+$24,270/呎
 (暂停销售)</t>
         </is>
       </c>
       <c r="J6" s="23" t="inlineStr">
         <is>
           <t>J | 354呎 (1房)
-$1069万
-$30,195/呎
+$855.12万
+$24,156/呎
 (暂停销售)</t>
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr">
         <is>
           <t>K | 380呎 (1房)
-$1108万
-$29,155/呎
+$886.32万
+$23,324/呎
 (暂停销售)</t>
         </is>
       </c>
@@ -81705,8 +81705,8 @@
       <c r="E11" s="20" t="inlineStr">
         <is>
           <t>D | 275呎 (开放式)
-$928万
-$33,745/呎
+$742.40万
+$26,996/呎
 (在售)</t>
         </is>
       </c>

</xml_diff>